<commit_message>
Industrial Optimization: 5-point traceability, simplified Roast Center, and demo assistant
</commit_message>
<xml_diff>
--- a/planillas_recoleccion/Planilla Maestra Axis Coffee Pro.xlsx
+++ b/planillas_recoleccion/Planilla Maestra Axis Coffee Pro.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FullStackDeveloper\axis-oil\axis_pro\planillas_recoleccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D5E84F-9459-4722-BCC4-7E70E6AFD808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C49E245A-6884-4B63-8922-C18587ABD3C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" firstSheet="1" activeTab="2" xr2:uid="{31E06617-1165-4898-AC29-7862C7F218B4}"/>
+    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" xr2:uid="{31E06617-1165-4898-AC29-7862C7F218B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilla_Maestra_AXIS_Integ (3)" sheetId="4" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="100">
   <si>
     <t>Fecha</t>
   </si>
@@ -159,9 +159,6 @@
     <t>Lote 2 (Equilibrio)</t>
   </si>
   <si>
-    <t>Lote 3 (Innovación)</t>
-  </si>
-  <si>
     <t>Luisa Fernanda G.</t>
   </si>
   <si>
@@ -222,9 +219,6 @@
     <t>18.2</t>
   </si>
   <si>
-    <t>22.0</t>
-  </si>
-  <si>
     <t>10.8</t>
   </si>
   <si>
@@ -258,9 +252,6 @@
     <t>Caramelo, Nuez</t>
   </si>
   <si>
-    <t>Frutas Rojas, Vino</t>
-  </si>
-  <si>
     <t>8.50</t>
   </si>
   <si>
@@ -285,14 +276,92 @@
     <t>Lote Comercial Premium</t>
   </si>
   <si>
-    <t>Perfil Exótico</t>
+    <t>Fecha de Recoleccion</t>
+  </si>
+  <si>
+    <t>Latitud</t>
+  </si>
+  <si>
+    <t>Longitud</t>
+  </si>
+  <si>
+    <t>Hectáreas</t>
+  </si>
+  <si>
+    <t>Agua ($A_W$)</t>
+  </si>
+  <si>
+    <t>Malla_15_Pct</t>
+  </si>
+  <si>
+    <t>Defectos_Primarios</t>
+  </si>
+  <si>
+    <t>Defectos_Secundarios</t>
+  </si>
+  <si>
+    <t>pH_Inicial</t>
+  </si>
+  <si>
+    <t>Grados Brix</t>
+  </si>
+  <si>
+    <t>Temperatura Masa</t>
+  </si>
+  <si>
+    <t>Envase de Fermentación</t>
+  </si>
+  <si>
+    <t>Duración Fermentación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fragancia </t>
+  </si>
+  <si>
+    <t>Frutas Rojas, Vino. Perfil Exótico</t>
+  </si>
+  <si>
+    <t>Postgusto</t>
+  </si>
+  <si>
+    <t>Global</t>
+  </si>
+  <si>
+    <t>Taza con Defectos</t>
+  </si>
+  <si>
+    <t>Catador / Q-Grader</t>
+  </si>
+  <si>
+    <t>Lote</t>
+  </si>
+  <si>
+    <t>Trilla</t>
+  </si>
+  <si>
+    <t>Laboratorio</t>
+  </si>
+  <si>
+    <t>Catación y perfilamiento de taza</t>
+  </si>
+  <si>
+    <t>Notas de Catación</t>
+  </si>
+  <si>
+    <t>Fermentación</t>
+  </si>
+  <si>
+    <t>Duración Secado</t>
+  </si>
+  <si>
+    <t>Tipo de Secado</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -326,8 +395,18 @@
       <sz val="9"/>
       <name val="Montserrat"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Montserrat"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Montserrat"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -338,6 +417,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor theme="9" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -403,17 +488,6 @@
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
@@ -462,47 +536,69 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -837,12 +933,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D73F090-8E81-436B-ADF5-84ED1602F3A5}">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17.55" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" style="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="28.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" style="13" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.77734375" bestFit="1" customWidth="1"/>
@@ -855,267 +951,401 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B1" s="3" t="s">
-        <v>34</v>
-      </c>
+      <c r="A1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="16"/>
     </row>
     <row r="2" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="5">
+        <v>45395</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8">
+        <v>1056784322</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B6" s="8"/>
+    </row>
+    <row r="7" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8">
+        <v>1920</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="8"/>
+    </row>
+    <row r="10" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="8"/>
+    </row>
+    <row r="11" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="17"/>
+    </row>
+    <row r="13" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="8"/>
+    </row>
+    <row r="14" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="8"/>
+    </row>
+    <row r="16" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="8"/>
+    </row>
+    <row r="17" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" s="8"/>
+    </row>
+    <row r="18" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B18" s="8"/>
+    </row>
+    <row r="19" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="17"/>
+    </row>
+    <row r="20" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" s="8"/>
+    </row>
+    <row r="23" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B23" s="8"/>
+    </row>
+    <row r="24" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A24" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" s="8">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="8">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A27" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A28" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="B29" s="17"/>
+    </row>
+    <row r="30" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A30" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" s="8">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B32" s="8"/>
+    </row>
+    <row r="33" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" s="8">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A35" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" s="8">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B36" s="8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B37" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A38" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" s="8">
         <v>0</v>
       </c>
-      <c r="B2" s="6">
-        <v>45395</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="9">
-        <v>1056784322</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="9">
-        <v>1920</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="9">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="9">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="9">
-        <v>730</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="9">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="9">
+    </row>
+    <row r="39" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A39" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A40" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B40" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A41" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B41" s="17"/>
+    </row>
+    <row r="42" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A42" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A43" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B19" s="9">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B20" s="9">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" s="9">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B22" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B25" s="9" t="s">
+      <c r="B43" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A44" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A45" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A46" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A47" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B47" s="8" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="7" t="s">
+    <row r="48" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A48" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B29" s="9" t="s">
+      <c r="B48" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A49" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A50" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B50" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="30.7" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="14" t="s">
-        <v>76</v>
-      </c>
+    <row r="51" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A51" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B51" s="15"/>
+    </row>
+    <row r="52" spans="1:2" ht="35.700000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B52" s="19" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A53" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="8"/>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A19:B19"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -1128,7 +1358,7 @@
   <cols>
     <col min="1" max="1" width="22.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="25.109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" style="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" style="13" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.77734375" bestFit="1" customWidth="1"/>
@@ -1146,259 +1376,259 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="4">
         <v>45395</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>36</v>
+      <c r="B3" s="7" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="7">
         <v>1109452331</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>39</v>
+      <c r="B5" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>42</v>
+      <c r="B6" s="7" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>45</v>
+      <c r="B7" s="7" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>48</v>
+      <c r="B8" s="7" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="7">
         <v>1650</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="7">
         <v>480</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="7">
         <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>51</v>
+      <c r="B12" s="7" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>54</v>
+      <c r="B13" s="7" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>57</v>
+      <c r="B14" s="7" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="7">
         <v>690</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="7">
         <v>388</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="7">
         <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="7">
         <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="7">
         <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="7">
         <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="7">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B22" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>60</v>
+      <c r="B23" s="7" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>63</v>
+      <c r="B24" s="7" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B26" s="8" t="s">
+    <row r="27" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A27" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A28" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A30" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B32" s="9" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B32" s="10" t="s">
+    <row r="33" spans="1:2" ht="30.7" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A33" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="12" t="s">
         <v>72</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="30.7" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1431,260 +1661,260 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="4">
         <v>45395</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="7">
+        <v>1081643221</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="7">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="7">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="7">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7">
+        <v>710</v>
+      </c>
+      <c r="F15" s="13"/>
+    </row>
+    <row r="16" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="7">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="7">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20" s="7">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="8">
-        <v>1081643221</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="20.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="8">
-        <v>1850</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="8">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="8">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="8">
-        <v>710</v>
-      </c>
-      <c r="F15" s="15"/>
-    </row>
-    <row r="16" spans="1:6" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="8">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="8">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B19" s="8">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="7" t="s">
+    <row r="21" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="7">
         <v>15</v>
       </c>
-      <c r="B20" s="8">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" s="8">
-        <v>15</v>
-      </c>
     </row>
     <row r="22" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B22" s="7">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>59</v>
+      <c r="B23" s="7" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>62</v>
+      <c r="B24" s="7" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B26" s="8" t="s">
+    <row r="27" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A27" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A28" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A30" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B32" s="9" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="18.2" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B32" s="10" t="s">
+    <row r="33" spans="1:2" ht="30.7" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A33" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="12" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="30.7" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>